<commit_message>
modification readme et notebook
</commit_message>
<xml_diff>
--- a/base_history_metriques_adam_train_val.xlsx
+++ b/base_history_metriques_adam_train_val.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/725bbd4577e01318/Desktop/MASTER_IA_DIT/DEVOIR_DEEP_LEARNING/cnn-catsdogs-DrameSekou/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_2B59D2BFD360D41BC101C8F050E0C0F37A01F933" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9FA1F51D-71BD-4540-A1B8-4BFEBEFB22F9}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_2B59D2BFD360D41BC101C8F050E0C0F37A01F933" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F5182D3-5A8B-4EF0-AA07-25F5BCF6A791}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -423,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.90625" bestFit="1" customWidth="1"/>
@@ -433,7 +433,7 @@
     <col min="8" max="8" width="11.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -459,7 +459,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -484,12 +484,8 @@
       <c r="H2" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J2">
-        <f>MAX(E2:E11)</f>
-        <v>0.7068888888888889</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -515,7 +511,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -541,7 +537,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -567,7 +563,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -593,7 +589,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -619,7 +615,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -645,7 +641,7 @@
         <v>1.0000000000000001E-5</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -671,7 +667,7 @@
         <v>1.0000000000000001E-5</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -697,7 +693,7 @@
         <v>1.0000000000000001E-5</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>10</v>
       </c>

</xml_diff>